<commit_message>
ya hice lo de excel
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -12,12 +12,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>Tarea</t>
   </si>
   <si>
     <t>gfdgdfg</t>
+  </si>
+  <si>
+    <t>ff</t>
+  </si>
+  <si>
+    <t>gdfg</t>
+  </si>
+  <si>
+    <t>f</t>
   </si>
 </sst>
 </file>
@@ -62,7 +71,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -75,6 +84,26 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
key enter and decoration in text field, and title bar move
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -12,18 +12,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Tarea</t>
   </si>
   <si>
-    <t>ff</t>
+    <t>asdasd</t>
   </si>
   <si>
-    <t>gdfg</t>
+    <t>knkjsnk</t>
   </si>
   <si>
-    <t>f</t>
+    <t>sadsad</t>
+  </si>
+  <si>
+    <t>absvdahsbjd</t>
+  </si>
+  <si>
+    <t>asbdjsnf</t>
   </si>
 </sst>
 </file>
@@ -68,7 +74,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -91,6 +97,16 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
i put the icon in the panels
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -12,9 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Tarea</t>
+  </si>
+  <si>
+    <t>hkj</t>
   </si>
 </sst>
 </file>
@@ -59,7 +62,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -67,6 +70,11 @@
         <v>0</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>